<commit_message>
Add Excel generation functionality for SQL conversion results
- Introduced a new script to generate Excel files containing conversion results from SQL statements.
- Implemented logic to extract relevant data from XML and format it for Excel output.
- Added support for handling various SQL operations (select, update, delete) and their corresponding parameters.
- Included test cases to validate the conversion process and ensure accurate output.
</commit_message>
<xml_diff>
--- a/IbatisToJdbcConverter_场景测试.xlsx
+++ b/IbatisToJdbcConverter_场景测试.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1565,10 +1565,14 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>测试找不到statement时抛出异常</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
+          <t>合并异常测试：</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>场景1：找不到 statementId</t>
+        </is>
+      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
           <t>mapOf("id", 1)</t>
@@ -1591,10 +1595,14 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>测试include引用不存在的sql片段时抛出异常</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
+          <t>合并异常测试：</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>场景2：include 引用不存在的 sql 片段</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
           <t>null</t>
@@ -1619,10 +1627,14 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>测试resultMap引用不存在的映射定义时抛出异常</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
+          <t>合并异常测试：</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>场景3：resultMap 引用不存在的映射定义</t>
+        </is>
+      </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
           <t>null</t>
@@ -1636,6 +1648,369 @@
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>场景1：parameterClass=long，传数字字符串 "123" -&gt; 应正确转换为 123L</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>"123"</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>SELECT id, name, status, created_at FROM users where id = 123</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>场景2：parameterClass=long，传数字 123 (Integer) -&gt; 应规范化为 123L (Long)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>SELECT id, name, status, created_at FROM users where id = 123</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>场景3：parameterClass=long，传非数字字符串 "not-a-number" -&gt; 应抛错</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>"not-a-number"</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>场景4：parameterClass=long，传空字符串 "" -&gt; 应抛错</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>""</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>场景5：parameterClass=long，传 boolean true -&gt; 应抛错</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>场景6：parameterClass=long，传 null -&gt; 应保留 null（不做转换）</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>SELECT id, name, status, created_at FROM users where id = null</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>场景7：parameterClass=string，传数字 12345 (Integer) -&gt; 应转为字符串 "12345"</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>12345</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersById" parameterClass="java.lang.String" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #Id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>SELECT id, name, status, created_at FROM users where id = '12345'</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>场景8：parameterClass=string，传 boolean true -&gt; 应转为字符串 "true"</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersById" parameterClass="java.lang.String" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #Id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>SELECT id, name, status, created_at FROM users where id = 'true'</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>场景9：parameterClass=map，传 List 时应抛错（集合类型不匹配）</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>listOf(1, 2, 3)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdMap" parameterClass="map" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>场景10：parameterClass=map，传 String 时应抛错（标量类型不匹配）</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>"not-a-map"</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdMap" parameterClass="map" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>综合测试：iBatis2 参数类型兼容性和转换规则</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>场景11：parameterClass=long，传 Map 时应抛错（完全不匹配）</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>mapOf("id", 123)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>&lt;select id="findUsersByIdNumber" parameterClass="java.lang.Long" resultClass="user"&gt;
+		SELECT id, name, status, created_at
+		FROM users where id = #id#
+	&lt;/select&gt;</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>